<commit_message>
Revise combat approach, attack cadence and projectile impacts
Use foot-space melee positioning, bounded ranged retreat, lifetime-safe hit timing, persistent first-owner taunts and boss-safe pulse control. Rebalance job and monster cadence through the existing catalog pipeline, block retired archer jobs, and add restrained pooled combat audio.

Validated with Unity 6000.3.21f1 Android IL2CPP, device melee/projectile samples and 18 live shield/taunt/control checks.
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Stage_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Stage_Catalog.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StageDefinitions" sheetId="1" r:id="R3555733e773349fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StageMonsters" sheetId="2" r:id="R7979abfec1fe4254"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MainBalance" sheetId="3" r:id="Rf73599a64989415e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GoldBalance" sheetId="4" r:id="R71969527c21840ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RubyBalance" sheetId="5" r:id="Rc753eaab6ac74304"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RubyRewards" sheetId="6" r:id="R452b683240914cb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FirstClearRewards" sheetId="7" r:id="Rc9f2f64002014d26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterCatalog" sheetId="8" r:id="R45662af79c114746"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnvironmentPresets" sheetId="9" r:id="R28af7f426231458b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KillCountFlow" sheetId="10" r:id="Re3d25a0d7a914464"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="11" r:id="Re3ead88ecccc4bbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="12" r:id="R92b67e09bc524bc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="13" r:id="R596d22029d4f4d8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="14" r:id="R392bcc74695346bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StageDefinitions" sheetId="1" r:id="R633c42b561ed426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StageMonsters" sheetId="2" r:id="Rfe014959acba4e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MainBalance" sheetId="3" r:id="Rce66d3bd61a540ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GoldBalance" sheetId="4" r:id="R7fb4273518334693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RubyBalance" sheetId="5" r:id="R73a7130cdddb4ebc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RubyRewards" sheetId="6" r:id="Rddf766057ee44427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FirstClearRewards" sheetId="7" r:id="Rcc09857d49464480"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterCatalog" sheetId="8" r:id="R37f594beb7dc412d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnvironmentPresets" sheetId="9" r:id="R00021399fa464dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KillCountFlow" sheetId="10" r:id="R985fd8f37665499a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="11" r:id="Rb45e5de0376d4892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="12" r:id="R1f9701cea6a44ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="13" r:id="R61b299d9b95d4aeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="14" r:id="R888ec767b3014e4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="8">
+  <x:numFmts count="9">
     <x:numFmt numFmtId="200" formatCode="#,##0;[Red]-#,##0;0"/>
     <x:numFmt numFmtId="201" formatCode="0.000"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
@@ -35,6 +35,7 @@
     <x:numFmt numFmtId="205" formatCode="0.0"/>
     <x:numFmt numFmtId="206" formatCode="0;&quot;—&quot;;0"/>
     <x:numFmt numFmtId="207" formatCode="0.00&quot;×&quot;"/>
+    <x:numFmt numFmtId="208" formatCode="0.00"/>
   </x:numFmts>
   <x:fonts count="10">
     <x:font>
@@ -105,7 +106,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -215,6 +216,10 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="208" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -452,8 +457,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Catalog_MonsterCatalog" displayName="Catalog_MonsterCatalog" ref="A1:J42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="Catalog_MonsterCatalog" displayName="Catalog_MonsterCatalog" ref="A1:K42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
     <x:tableColumn id="1" name="MonsterName"/>
     <x:tableColumn id="2" name="MonsterId"/>
     <x:tableColumn id="3" name="DisplayName"/>
@@ -464,6 +469,7 @@
     <x:tableColumn id="8" name="MoveSpeed"/>
     <x:tableColumn id="9" name="AttackIntervalSec"/>
     <x:tableColumn id="10" name="Notes"/>
+    <x:tableColumn id="11" name="AttackMultiplier"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -3017,7 +3023,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0e3b117d60d4c41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a3aadff3f014e82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3091,7 +3097,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R505b79967023479d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7994c0a343864619"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3868,7 +3874,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R344e1d89df8a4ba7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99e29c76d4c34c76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14912,7 +14918,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca2e2d6920c644d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a65c8384e1f49d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15110,7 +15116,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra51ad940ef1d460f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e50096887174c61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15297,7 +15303,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R346bbeb604414d93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c51d1b4448c4adc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19735,7 +19741,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb916650544a24efe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R434a50ca26694089"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21831,7 +21837,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6aaa77672374e0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb669e2c1d2c94b05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22147,7 +22153,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4461cfc1a064fd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf9b53b7b06e4a86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22222,7 +22228,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G2" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="H2" s="19" t="str">
         <x:v>면역</x:v>
@@ -22254,7 +22260,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G3" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H3" s="19" t="str">
         <x:v>면역</x:v>
@@ -22286,7 +22292,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G4" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="H4" s="19" t="str">
         <x:v>면역</x:v>
@@ -22318,7 +22324,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G5" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="H5" s="19" t="str">
         <x:v>면역</x:v>
@@ -22350,7 +22356,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G6" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H6" s="19" t="str">
         <x:v>면역</x:v>
@@ -22382,7 +22388,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G7" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="H7" s="19" t="str">
         <x:v>면역</x:v>
@@ -22414,7 +22420,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G8" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="H8" s="19" t="str">
         <x:v>면역</x:v>
@@ -22446,7 +22452,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G9" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H9" s="19" t="str">
         <x:v>면역</x:v>
@@ -22478,7 +22484,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G10" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="H10" s="19" t="str">
         <x:v>면역</x:v>
@@ -22510,7 +22516,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G11" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="H11" s="19" t="str">
         <x:v>면역</x:v>
@@ -22542,7 +22548,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G12" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
         <x:v>면역</x:v>
@@ -22574,7 +22580,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G13" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="H13" s="19" t="str">
         <x:v>면역</x:v>
@@ -22606,7 +22612,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G14" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="H14" s="19" t="str">
         <x:v>면역</x:v>
@@ -22638,7 +22644,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G15" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H15" s="19" t="str">
         <x:v>면역</x:v>
@@ -22670,7 +22676,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="G16" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="H16" s="19" t="str">
         <x:v>면역</x:v>
@@ -22682,7 +22688,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R285f6f59219841d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17902bd1f5fd4d66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22864,7 +22870,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68d2bfe8f9b44b81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91c362dd8df9446e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23251,7 +23257,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd561a7c7a3434dbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56b6cf894cc0425c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23273,6 +23279,7 @@
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="70" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="43" customHeight="1">
@@ -23306,6 +23313,9 @@
       <x:c r="J1" s="18" t="str">
         <x:v>Notes</x:v>
       </x:c>
+      <x:c r="K1" t="str">
+        <x:v>AttackMultiplier</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
       <x:c r="A2" s="19" t="str">
@@ -23330,13 +23340,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/Bat.prefab</x:v>
       </x:c>
       <x:c r="H2" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I2" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I2" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="J2" s="19" t="str">
         <x:v>Attack source absent; visual fallback Walk (content-specific behavior remains future work); Hurt source absent; visual fallback Idle (content-specific behavior remains future work); Dead source absent; visual fallback Transform (content-specific behavior remains future work)</x:v>
+      </x:c>
+      <x:c r="K2" s="31" t="n">
+        <x:v>0.8</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
@@ -23362,12 +23375,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/Bugbear.prefab</x:v>
       </x:c>
       <x:c r="H3" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I3" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="I3" s="32" t="n">
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="J3" s="19" t="str"/>
+      <x:c r="K3" s="31" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
       <x:c r="A4" s="19" t="str">
@@ -23392,12 +23408,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Dragons/ElderDragon.prefab</x:v>
       </x:c>
       <x:c r="H4" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I4" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J4" s="19" t="str"/>
+      <x:c r="K4" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I4" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J4" s="19" t="str"/>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
       <x:c r="A5" s="19" t="str">
@@ -23422,12 +23441,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Dragons/ElderDragonBlue.prefab</x:v>
       </x:c>
       <x:c r="H5" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I5" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J5" s="19" t="str"/>
+      <x:c r="K5" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I5" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J5" s="19" t="str"/>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="19" t="str">
@@ -23452,12 +23474,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Dragons/ElderDragonGray.prefab</x:v>
       </x:c>
       <x:c r="H6" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I6" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J6" s="19" t="str"/>
+      <x:c r="K6" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I6" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J6" s="19" t="str"/>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="19" t="str">
@@ -23482,12 +23507,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Dragons/ElderDragonGreen.prefab</x:v>
       </x:c>
       <x:c r="H7" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I7" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J7" s="19" t="str"/>
+      <x:c r="K7" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I7" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J7" s="19" t="str"/>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="19" t="str">
@@ -23512,12 +23540,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Dragons/ElderDragonOrange.prefab</x:v>
       </x:c>
       <x:c r="H8" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I8" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J8" s="19" t="str"/>
+      <x:c r="K8" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I8" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J8" s="19" t="str"/>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="19" t="str">
@@ -23542,12 +23573,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Dragons/ElderDragonPink.prefab</x:v>
       </x:c>
       <x:c r="H9" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I9" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J9" s="19" t="str"/>
+      <x:c r="K9" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I9" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J9" s="19" t="str"/>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="19" t="str">
@@ -23572,12 +23606,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Dragons/ElderDragonPurple.prefab</x:v>
       </x:c>
       <x:c r="H10" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I10" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J10" s="19" t="str"/>
+      <x:c r="K10" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I10" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J10" s="19" t="str"/>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="19" t="str">
@@ -23602,12 +23639,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Dragons/ElderDragonRed.prefab</x:v>
       </x:c>
       <x:c r="H11" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I11" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J11" s="19" t="str"/>
+      <x:c r="K11" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I11" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J11" s="19" t="str"/>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="19" t="str">
@@ -23632,12 +23672,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Dragons/ElderDragonYellow.prefab</x:v>
       </x:c>
       <x:c r="H12" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I12" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J12" s="19" t="str"/>
+      <x:c r="K12" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I12" s="19" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J12" s="19" t="str"/>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="19" t="str">
@@ -23662,13 +23705,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/Frog.prefab</x:v>
       </x:c>
       <x:c r="H13" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I13" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I13" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="J13" s="19" t="str">
         <x:v>Attack source absent; visual fallback Walk (content-specific behavior remains future work); Hurt source absent; visual fallback Idle (content-specific behavior remains future work); Dead source absent; visual fallback Transform (content-specific behavior remains future work)</x:v>
+      </x:c>
+      <x:c r="K13" s="31" t="n">
+        <x:v>0.8</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
@@ -23694,12 +23740,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/Goblin.prefab</x:v>
       </x:c>
       <x:c r="H14" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I14" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I14" s="32" t="n">
+        <x:v>1.35</x:v>
       </x:c>
       <x:c r="J14" s="19" t="str"/>
+      <x:c r="K14" s="31" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="19" t="str">
@@ -23724,12 +23773,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/GoblinAssassin.prefab</x:v>
       </x:c>
       <x:c r="H15" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I15" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="I15" s="32" t="n">
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="J15" s="19" t="str"/>
+      <x:c r="K15" s="31" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="19" t="str">
@@ -23754,12 +23806,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/GoblinBoarRider.prefab</x:v>
       </x:c>
       <x:c r="H16" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I16" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I16" s="32" t="n">
+        <x:v>1.75</x:v>
       </x:c>
       <x:c r="J16" s="19" t="str"/>
+      <x:c r="K16" s="31" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="19" t="str">
@@ -23784,12 +23839,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/GoblinBomber.prefab</x:v>
       </x:c>
       <x:c r="H17" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I17" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="I17" s="32" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J17" s="19" t="str"/>
+      <x:c r="K17" s="31" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="19" t="str">
@@ -23814,12 +23872,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/GoblinGunner.prefab</x:v>
       </x:c>
       <x:c r="H18" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I18" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I18" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="J18" s="19" t="str"/>
+      <x:c r="K18" s="31" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="19" t="str">
@@ -23844,12 +23905,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/GoblinKamikaze.prefab</x:v>
       </x:c>
       <x:c r="H19" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I19" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I19" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="J19" s="19" t="str"/>
+      <x:c r="K19" s="31" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="19" t="str">
@@ -23874,12 +23938,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/GoblinKing.prefab</x:v>
       </x:c>
       <x:c r="H20" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I20" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="I20" s="32" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J20" s="19" t="str"/>
+      <x:c r="K20" s="31" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
       <x:c r="A21" s="19" t="str">
@@ -23904,12 +23971,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/GoblinMechRider.prefab</x:v>
       </x:c>
       <x:c r="H21" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I21" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="I21" s="32" t="n">
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="J21" s="19" t="str"/>
+      <x:c r="K21" s="31" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="19" t="str">
@@ -23934,12 +24004,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/GoblinShaman.prefab</x:v>
       </x:c>
       <x:c r="H22" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I22" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="I22" s="32" t="n">
+        <x:v>1.85</x:v>
       </x:c>
       <x:c r="J22" s="19" t="str"/>
+      <x:c r="K22" s="31" t="n">
+        <x:v>1.05</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" s="19" t="str">
@@ -23964,12 +24037,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/GoblinWorker.prefab</x:v>
       </x:c>
       <x:c r="H23" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I23" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I23" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="J23" s="19" t="str"/>
+      <x:c r="K23" s="31" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
       <x:c r="A24" s="19" t="str">
@@ -23994,12 +24070,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Mimics/HeresyMimic.prefab</x:v>
       </x:c>
       <x:c r="H24" s="22" t="n">
-        <x:v>1.2</x:v>
-      </x:c>
-      <x:c r="I24" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="I24" s="32" t="n">
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="J24" s="19" t="str"/>
+      <x:c r="K24" s="31" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
       <x:c r="A25" s="19" t="str">
@@ -24024,13 +24103,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/Goblins/LootGoblin.prefab</x:v>
       </x:c>
       <x:c r="H25" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I25" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I25" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="J25" s="19" t="str">
         <x:v>Attack source absent; visual fallback Walk (content-specific behavior remains future work)</x:v>
+      </x:c>
+      <x:c r="K25" s="31" t="n">
+        <x:v>0.8</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
@@ -24056,13 +24138,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/Mimics/MimicBarrel.prefab</x:v>
       </x:c>
       <x:c r="H26" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I26" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I26" s="32" t="n">
+        <x:v>1.75</x:v>
       </x:c>
       <x:c r="J26" s="19" t="str">
         <x:v>Source pack has no dedicated Hurt/Dead rows; prepared Hurt uses one idle pose, Dead closes the container (reverse Reveal; Sack settles to idle). No new behavior is implemented.</x:v>
+      </x:c>
+      <x:c r="K26" s="31" t="n">
+        <x:v>1.1</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
@@ -24088,13 +24173,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/Mimics/MimicChest.prefab</x:v>
       </x:c>
       <x:c r="H27" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I27" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I27" s="32" t="n">
+        <x:v>1.75</x:v>
       </x:c>
       <x:c r="J27" s="19" t="str">
         <x:v>Source pack has no dedicated Hurt/Dead rows; prepared Hurt uses one idle pose, Dead closes the container (reverse Reveal; Sack settles to idle). No new behavior is implemented.</x:v>
+      </x:c>
+      <x:c r="K27" s="31" t="n">
+        <x:v>1.1</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
@@ -24120,13 +24208,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/Mimics/MimicSack.prefab</x:v>
       </x:c>
       <x:c r="H28" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I28" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I28" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="J28" s="19" t="str">
         <x:v>Source pack has no dedicated Hurt/Dead rows; prepared Hurt uses one idle pose, Dead closes the container (reverse Reveal; Sack settles to idle). No new behavior is implemented.</x:v>
+      </x:c>
+      <x:c r="K28" s="31" t="n">
+        <x:v>0.8</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
@@ -24152,12 +24243,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/OrcBrute.prefab</x:v>
       </x:c>
       <x:c r="H29" s="22" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="I29" s="32" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="J29" s="19" t="str"/>
+      <x:c r="K29" s="31" t="n">
         <x:v>1.5</x:v>
       </x:c>
-      <x:c r="I29" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="J29" s="19" t="str"/>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
       <x:c r="A30" s="19" t="str">
@@ -24182,12 +24276,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/OrcHunter.prefab</x:v>
       </x:c>
       <x:c r="H30" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I30" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.05</x:v>
+      </x:c>
+      <x:c r="I30" s="32" t="n">
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J30" s="19" t="str"/>
+      <x:c r="K30" s="31" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="25" customHeight="1">
       <x:c r="A31" s="19" t="str">
@@ -24212,12 +24309,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/OrcKamikaze.prefab</x:v>
       </x:c>
       <x:c r="H31" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I31" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I31" s="32" t="n">
+        <x:v>1.75</x:v>
       </x:c>
       <x:c r="J31" s="19" t="str"/>
+      <x:c r="K31" s="31" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="25" customHeight="1">
       <x:c r="A32" s="19" t="str">
@@ -24242,13 +24342,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/OrcKid.prefab</x:v>
       </x:c>
       <x:c r="H32" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I32" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I32" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="J32" s="19" t="str">
         <x:v>Hurt source absent; visual fallback Cry (content-specific behavior remains future work); Dead source absent; visual fallback Cry (content-specific behavior remains future work)</x:v>
+      </x:c>
+      <x:c r="K32" s="31" t="n">
+        <x:v>0.8</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="25" customHeight="1">
@@ -24274,12 +24377,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/OrcPeon.prefab</x:v>
       </x:c>
       <x:c r="H33" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I33" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I33" s="32" t="n">
+        <x:v>1.75</x:v>
       </x:c>
       <x:c r="J33" s="19" t="str"/>
+      <x:c r="K33" s="31" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="25" customHeight="1">
       <x:c r="A34" s="19" t="str">
@@ -24304,12 +24410,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/OrcShaman.prefab</x:v>
       </x:c>
       <x:c r="H34" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I34" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I34" s="32" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J34" s="19" t="str"/>
+      <x:c r="K34" s="31" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="25" customHeight="1">
       <x:c r="A35" s="19" t="str">
@@ -24334,12 +24443,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/OrcTaskmaster.prefab</x:v>
       </x:c>
       <x:c r="H35" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I35" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="I35" s="32" t="n">
+        <x:v>2.15</x:v>
       </x:c>
       <x:c r="J35" s="19" t="str"/>
+      <x:c r="K35" s="31" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="25" customHeight="1">
       <x:c r="A36" s="19" t="str">
@@ -24364,12 +24476,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/OrcWarlock.prefab</x:v>
       </x:c>
       <x:c r="H36" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I36" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="I36" s="32" t="n">
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="J36" s="19" t="str"/>
+      <x:c r="K36" s="31" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="25" customHeight="1">
       <x:c r="A37" s="19" t="str">
@@ -24394,12 +24509,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/OrcWarrior.prefab</x:v>
       </x:c>
       <x:c r="H37" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I37" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="I37" s="32" t="n">
+        <x:v>1.85</x:v>
       </x:c>
       <x:c r="J37" s="19" t="str"/>
+      <x:c r="K37" s="31" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="25" customHeight="1">
       <x:c r="A38" s="19" t="str">
@@ -24424,12 +24542,15 @@
         <x:v>Assets/_Project/Prefabs/Monster/Orcs/Quasit.prefab</x:v>
       </x:c>
       <x:c r="H38" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I38" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="I38" s="32" t="n">
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="J38" s="19" t="str"/>
+      <x:c r="K38" s="31" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="25" customHeight="1">
       <x:c r="A39" s="19" t="str">
@@ -24454,13 +24575,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/BANDIT/MON_BANDIT_ARCHER.prefab</x:v>
       </x:c>
       <x:c r="H39" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I39" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="I39" s="32" t="n">
+        <x:v>1.7</x:v>
       </x:c>
       <x:c r="J39" s="19" t="str">
         <x:v>기존 ID·프리팹 유지</x:v>
+      </x:c>
+      <x:c r="K39" s="31" t="n">
+        <x:v>0.95</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="25" customHeight="1">
@@ -24486,13 +24610,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/BANDIT/MON_BANDIT_LEADER.prefab</x:v>
       </x:c>
       <x:c r="H40" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I40" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="I40" s="32" t="n">
+        <x:v>1.6</x:v>
       </x:c>
       <x:c r="J40" s="19" t="str">
         <x:v>기존 ID·프리팹 유지</x:v>
+      </x:c>
+      <x:c r="K40" s="31" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="25" customHeight="1">
@@ -24518,13 +24645,16 @@
         <x:v>Assets/_Project/Prefabs/Monster/BANDIT/MON_BANDIT_SHIELD.prefab</x:v>
       </x:c>
       <x:c r="H41" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I41" s="19" t="n">
-        <x:v>1</x:v>
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="I41" s="32" t="n">
+        <x:v>1.95</x:v>
       </x:c>
       <x:c r="J41" s="19" t="str">
         <x:v>기존 ID·프리팹 유지</x:v>
+      </x:c>
+      <x:c r="K41" s="31" t="n">
+        <x:v>1.15</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="25" customHeight="1">
@@ -24550,19 +24680,22 @@
         <x:v>Assets/_Project/Prefabs/Monster/BANDIT/BANDIT_KING.prefab</x:v>
       </x:c>
       <x:c r="H42" s="22" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="I42" s="22" t="n">
-        <x:v>1.5</x:v>
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="I42" s="32" t="n">
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="J42" s="19" t="str">
         <x:v>기존 ID·프리팹 유지</x:v>
+      </x:c>
+      <x:c r="K42" s="31" t="n">
+        <x:v>1.35</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf15ad09520f4af4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba77cd8cd6ff4124"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26405,7 +26538,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra488ac0ff60c4728"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ec8c887b6704826"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(progression): continue chapters beyond three and return from dungeons on a visible timer
</commit_message>
<xml_diff>
--- a/Assets/_Project/Scripts/Stage_Catalog.xlsx
+++ b/Assets/_Project/Scripts/Stage_Catalog.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StageDefinitions" sheetId="1" r:id="R633c42b561ed426c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StageMonsters" sheetId="2" r:id="Rfe014959acba4e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MainBalance" sheetId="3" r:id="Rce66d3bd61a540ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GoldBalance" sheetId="4" r:id="R7fb4273518334693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RubyBalance" sheetId="5" r:id="R73a7130cdddb4ebc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RubyRewards" sheetId="6" r:id="Rddf766057ee44427"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FirstClearRewards" sheetId="7" r:id="Rcc09857d49464480"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterCatalog" sheetId="8" r:id="R37f594beb7dc412d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnvironmentPresets" sheetId="9" r:id="R00021399fa464dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KillCountFlow" sheetId="10" r:id="R985fd8f37665499a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="11" r:id="Rb45e5de0376d4892"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="12" r:id="R1f9701cea6a44ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="13" r:id="R61b299d9b95d4aeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="14" r:id="R888ec767b3014e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StageDefinitions" sheetId="1" r:id="Rc62eb4cbc8bd4e43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StageMonsters" sheetId="2" r:id="R57f7391c14f742e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MainBalance" sheetId="3" r:id="R2e04f3b3a3ce4d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GoldBalance" sheetId="4" r:id="R321cdbd962854227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RubyBalance" sheetId="5" r:id="R69a82f2fe5d943f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RubyRewards" sheetId="6" r:id="Rc11927b83f954f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FirstClearRewards" sheetId="7" r:id="R4215a5ffaa57451a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterCatalog" sheetId="8" r:id="R4febbb997d03498d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EnvironmentPresets" sheetId="9" r:id="R9a4a72c5cbd3439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KillCountFlow" sheetId="10" r:id="Rdcfe1b686dbf4cc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="11" r:id="Rf92751e215564ea3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth" sheetId="12" r:id="Ra9b6114ea84f4b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="13" r:id="Rbbdd68d0665349b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="14" r:id="R21022588aad54a92"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="9">
+  <x:numFmts count="10">
     <x:numFmt numFmtId="200" formatCode="#,##0;[Red]-#,##0;0"/>
     <x:numFmt numFmtId="201" formatCode="0.000"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
@@ -36,8 +36,9 @@
     <x:numFmt numFmtId="206" formatCode="0;&quot;—&quot;;0"/>
     <x:numFmt numFmtId="207" formatCode="0.00&quot;×&quot;"/>
     <x:numFmt numFmtId="208" formatCode="0.00"/>
+    <x:numFmt numFmtId="209" formatCode="0.##"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -86,8 +87,18 @@
       <x:color rgb="FF254E8A"/>
       <x:name val="Malgun Gothic"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF24374B"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1763B1"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -99,6 +110,16 @@
         <x:fgColor rgb="FF253E52"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF3FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF3FF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -106,7 +127,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -221,6 +242,13 @@
     <x:xf numFmtId="208" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="209" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="11" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -3023,7 +3051,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a3aadff3f014e82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23b3015bd1024e4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3071,7 +3099,7 @@
         <x:v>Any</x:v>
       </x:c>
       <x:c r="D2" s="19" t="str">
-        <x:v>ReturnToMainStage</x:v>
+        <x:v>AwaitDefeatChoice</x:v>
       </x:c>
       <x:c r="E2" s="19" t="str">
         <x:v>5체씩 4묶음, 처치 보상은 실패해도 보존</x:v>
@@ -3088,7 +3116,7 @@
         <x:v>Any</x:v>
       </x:c>
       <x:c r="D3" s="19" t="str">
-        <x:v>ReturnToMainStage</x:v>
+        <x:v>AwaitDefeatChoice</x:v>
       </x:c>
       <x:c r="E3" s="19" t="str">
         <x:v>3보스 순차, 각 30초·전환 0.8초 동안 시간 정지</x:v>
@@ -3097,7 +3125,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7994c0a343864619"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07eb2da214a04d4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3871,10 +3899,94 @@
         <x:v>민감도: EXP 획득 강화 현재 L</x:v>
       </x:c>
     </x:row>
+    <x:row r="55" ht="32" customHeight="1">
+      <x:c r="A55" s="34" t="str">
+        <x:v>endlessHpPower</x:v>
+      </x:c>
+      <x:c r="B55" s="39" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C55" s="34" t="str">
+        <x:v>지수</x:v>
+      </x:c>
+      <x:c r="D55" s="34" t="str">
+        <x:v>34번째 구간부터: 33구간 일반 HP × (진행번호/33)^지수</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="32" customHeight="1">
+      <x:c r="A56" s="34" t="str">
+        <x:v>endlessAtkPower</x:v>
+      </x:c>
+      <x:c r="B56" s="39" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C56" s="34" t="str">
+        <x:v>지수</x:v>
+      </x:c>
+      <x:c r="D56" s="34" t="str">
+        <x:v>이후 공격 성장; 몬스터별 역할 계수 유지</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="32" customHeight="1">
+      <x:c r="A57" s="34" t="str">
+        <x:v>endlessGoldPower</x:v>
+      </x:c>
+      <x:c r="B57" s="39" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="C57" s="34" t="str">
+        <x:v>지수</x:v>
+      </x:c>
+      <x:c r="D57" s="34" t="str">
+        <x:v>이후 골드 성장; 보스 배율은 기존 Inputs 적용</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="32" customHeight="1">
+      <x:c r="A58" s="34" t="str">
+        <x:v>endlessExpPower</x:v>
+      </x:c>
+      <x:c r="B58" s="39" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="C58" s="34" t="str">
+        <x:v>지수</x:v>
+      </x:c>
+      <x:c r="D58" s="34" t="str">
+        <x:v>이후 경험치 성장; 기존 계정 레벨 상한 유지</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="32" customHeight="1">
+      <x:c r="A59" s="34" t="str">
+        <x:v>endlessBossCoins</x:v>
+      </x:c>
+      <x:c r="B59" s="39" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C59" s="34" t="str">
+        <x:v>주화/장</x:v>
+      </x:c>
+      <x:c r="D59" s="34" t="str">
+        <x:v>4장 이후 보스 최초 완료 시; 계정당 해당 장 1회</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="32" customHeight="1">
+      <x:c r="A60" s="34" t="str">
+        <x:v>endlessBossFragments</x:v>
+      </x:c>
+      <x:c r="B60" s="39" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C60" s="34" t="str">
+        <x:v>전직 파편/장</x:v>
+      </x:c>
+      <x:c r="D60" s="34" t="str">
+        <x:v>4장 이후 보스 최초 완료 시; 환생 후 중복 지급 없음</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99e29c76d4c34c76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aa0b42470cd43be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14918,7 +15030,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a65c8384e1f49d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc987f0864ed6438e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15116,7 +15228,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e50096887174c61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f4847a657d64d79"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15303,7 +15415,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c51d1b4448c4adc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R000cedcdf6a84122"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19741,7 +19853,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R434a50ca26694089"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3c1aff38bff4f39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21837,7 +21949,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb669e2c1d2c94b05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R544c0e0228dd48c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22153,7 +22265,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf9b53b7b06e4a86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd5adc78c54349ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22688,7 +22800,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17902bd1f5fd4d66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6beddd802ae249e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22870,7 +22982,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91c362dd8df9446e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf203429704b840ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23257,7 +23369,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56b6cf894cc0425c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68d903155b794ea1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24695,7 +24807,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba77cd8cd6ff4124"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e0e8b9609474f9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26538,7 +26650,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ec8c887b6704826"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a2b2b41e24a4c48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>